<commit_message>
107th Commit: Epic Seven Completed
</commit_message>
<xml_diff>
--- a/EPIC_0005_Ride_Safety_Calls.xlsx
+++ b/EPIC_0005_Ride_Safety_Calls.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372B66B2-0197-40A5-94BD-8AADFE3B486B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66346BB1-D980-40E5-BC74-7E1A9DFEFE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
     <sheet name="CustomerAppEmergencyNumber" sheetId="48" r:id="rId2"/>
+    <sheet name="PanicCallCheck" sheetId="49" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -411,6 +412,280 @@
   </si>
   <si>
     <t>TC_RG_01_Emergency_Calls</t>
+  </si>
+  <si>
+    <t>Panic Call Check</t>
+  </si>
+  <si>
+    <t>TC_RG_02_Panic_Call</t>
+  </si>
+  <si>
+    <t>1. Reload the User App completely.
+2. Reload the Driver App completely.
+3. Switch to the Super Admin Web Portal session.
+4. Click on "Dashboard" from the navigation menu.
+5. Click on "Settings" in the navigation menu.
+6. Click on "Panic Call Setting" from the sidebar menu.
+7. Click the "Add Panic Call" button.
+8. Enter the name (Police) into the name input field.
+9. Enter the name in Tamil (காவல்துறை) into the Tamil name input field.
+10. Enter the name in Hindi (पुलिस) into the Hindi name input field.
+11. Enter the contact number (100) into the contact number field.
+12. Click the Status dropdown.
+13. Select "Active" from the status dropdown options.
+14. Click the "Submit" button to save the panic call setting.
+15. Search for the created panic call entry using the name.
+16. Wait 1 second for the search results to load.
+17. Switch to the Driver App session.
+18. Wait for the notification permission dialog to appear.
+19. Tap "Allow" to grant notification permissions.
+20. Set the mock location of the Driver device to Perambur (Coordinates: 13.121030, 80.232578).
+21. Tap "Agree" on the terms and conditions screen.
+22. Tap "Get Started" on the onboarding screen.
+23. Tap "Next" to navigate through onboarding.
+24. Tap the Mobile Number input field.
+25. Tap "Close" to dismiss any system auto-fill popups.
+26. Enter the approved driver mobile number.
+27. Wait for the "Continue" button to become visible.
+28. Tap "Continue".
+29. Enter the verification OTP (123456).
+30. Tap "Allow" to grant location permissions.
+31. Wait for the Driver App home header label to display.
+32. Wait 3 seconds for the Driver App status toggle to turn ON.
+33. Wait an additional 2 seconds to ensure driver online status is active.
+34. Switch back to the User App session.
+35. Wait for the "Get Started" button to display on the User App screen.
+36. Tap "Get Started".
+37. Tap "Allow" to grant notification permissions.
+38. Set the mock location of the User device to Perambur (Coordinates: 13.121030, 80.232578).
+39. Tap "Next".
+40. Tap the Mobile Number input field.
+41. Tap "Close" to dismiss any system auto-fill popups.
+42. Enter the customer mobile number.
+43. Wait for the "Continue" button to become visible.
+44. Tap "Continue".
+45. Enter the verification OTP (123456).
+46. Wait for the "Finish" button to become visible.
+47. Tap "Finish".
+48. Tap "Allow" to grant location permissions.
+49. Wait for the "Auto Ride" option to display on the home screen.
+50. Tap "Auto Ride".
+51. Enter the destination address ("Parsn Manare") into the destination search field.
+52. Wait for the location map selection screen to load.
+53. Tap the first destination suggestion from the search results.
+54. Wait for the entrance location selector to display.
+55. Tap the entrance location option.
+56. Tap "Confirm" to set the destination.
+57. Wait 5 seconds for ride estimation and vehicle availability.
+58. Wait for the "Ride Now" button to become visible.
+59. Tap "Ride Now" to request a booking.
+60. Switch to the Driver App session.
+61. Wait for the ride request notification and Accept button to display.
+62. Tap "Accept Ride" to confirm the booking.
+63. Switch to the User App session.
+64. Wait for the ride OTP display element to load on screen.
+65. Note down/Extract the displayed ride OTP from the screen.
+66. Wait 2 seconds for the ride interface to stabilize.
+67. Tap the "SOS" button on the active ride screen.
+68. Tap the "Police" button from the emergency options.
+69. Tap the "Call" button to initiate the emergency panic call.
+70. Wait 6 seconds for the emergency call action to process and return.
+71. Switch to the User App session.
+72. Switch to the Driver App session.
+73. Wait for the "On My Way" status button to display.
+74. Wait for the "Arrived" status button to display.
+75. Ensure the "Arrived" status button is fully visible.
+76. Tap "Arrived" to update driver arrival status.
+77. Wait for the confirmation dialog button ("Yes") to appear.
+78. Tap "Yes" to confirm arrival.
+79. Wait for the "Start Ride" button to display.
+80. Tap "Start Ride".
+81. Wait for the OTP input field to display.
+82. Enter the extracted ride OTP into the OTP input field.
+83. Wait for the "Start" button to become visible.
+84. Tap the "Start" button to commence the trip.
+85. Wait 3 seconds for the trip to register as started.
+86. Tap the "SOS" button using coordinates (972, 1207).
+87. Tap the "Police / 108 Call" option.
+88. Tap the "Call" button to initiate the panic call from the driver app.
+89. Wait 5 seconds for the phone dialer interface to interact/return.
+90. Switch to the Driver App session.
+91. Wait for the "Complete Ride" button to display.
+92. Tap "Complete Ride".
+93. Wait for the "Collect Payment" button to display.
+94. Tap "Collect Payment".
+95. Switch to the User App session.
+96. Wait for the "Proceed to Pay" button to display.
+97. Tap "Proceed to Pay".
+98. Wait for the payment confirmation option to display.
+99. Tap "Pay Cash" to choose cash as the payment method.
+100. Wait for the "Give Review" screen/button to display.
+101. Tap "Give Review".
+102. Tap the rating stars at coordinates (348, 1619) to set rating.
+103. Tap "Submit Rating".
+104. Wait for the "Done" button to appear.
+105. Tap "Done" to finish the ride process on the customer app.
+106. Switch to the Driver App session.
+107. Wait for the payment "Proceed" button to display.
+108. Tap "Proceed".
+109. Wait for the "Yes" confirmation button to appear.
+110. Tap "Yes" to confirm receipt of payment.
+111. Wait for the "Give Review" button to display.
+112. Tap "Give Review".
+113. Wait 2 seconds for the rating screen to load.
+114. Tap the rating stars at coordinates (348, 1545) to set rating.
+115. Tap "Submit Rating".
+116. Wait for the "Complete" button to display.
+117. Tap "Complete".
+118. Wait for the final ride complete submit button to display.
+119. Tap "Ride Complete Submit".
+120. Switch to the Super Admin Web Portal session.
+121. Click on "Dashboard" from the navigation menu.
+122. Click on "Settings" in the navigation menu.
+123. Click on "Panic Call Setting" from the sidebar menu.
+124. Search for the created panic call entry using the name.
+125. Wait 1 second for search results to load.
+126. Click the "Delete" button for the panic call entry.
+127. Click "Confirm Delete" on the confirmation modal.
+128. Wait 2 seconds for deletion process to complete.</t>
+  </si>
+  <si>
+    <t>This test case validates the end-to-end integration and execution of the Panic Call (SOS) feature across the Super Admin Web Portal, User App, and Driver App during an active Auto Ride session. It covers creating and activating a multilingual emergency contact (Police - 100) in the Admin Portal, configuring driver and customer locations in Perambur, requesting and accepting an Auto Ride, and extracting the OTP to start the trip. It verifies that both customer and driver can successfully trigger the SOS button and initiate emergency police calls during the ride, and completes the flow by processing cash payment, exchanging mutual user-driver reviews, and cleaning up the test data by deleting the panic contact in the Super Admin Portal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin Web portal is accessible and Cutomer and Driver App is availbale in emulator </t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3. Switch To Web,switch_to,web,
+4. Click Dashboard,Click,,"web.global.menu.dashboard"
+5. Click Setting,click,,"admin.setting.sidebar.menu"
+6. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+7. Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
+8. Enter name,type,Police&gt;&gt;policeName,"admin.setting.panic_call.name_input"
+9. Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
+10. Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
+11. Contact number,type,100,"admin.setting.panic_call.contact_number"
+12. Select Status button,click,,"admin.setting.panic_call.status_dropdown"
+13. Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
+14. Submit button,click,,"web.global.action.submit"
+15. Search name,type,{policeName},"admin.setting.panic_call.search_name"
+16. Wait For Load,wait,1000,
+17. Load Driver App,switch_to,driver,
+18. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+19. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+20. Force Driver Location To Perambur,set_location,13.121030;80.232578,
+21. Click Agree,tap,,"mobile.driver.agree.btn"
+22. Click Get Started,tap,,"mobile.driver.get_started.btn"
+23. Click Next,tap,,"mobile.driver.next.btn"
+24. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+25. Click Close,tap,,"mobile.driver.cancel.btn"
+26. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+27. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+28. Click Continue,tap,,"mobile.driver.continue.btn"
+29. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+30. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+31. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+32. Wait For Driver App Toggle On,wait,3000,
+33. Wait For Driver App Toggle On,wait,2000, 
+34. Load User App,switch_to,user,
+35. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+36. Click Get Started,tap,,"mobile.customer.get_started.btn"
+37. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+38. Force User Location To Perambur,set_location,13.121030;80.232578,
+39. Click Next,tap,,"mobile.customer.next.btn"
+40. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+41. Click Close,tap,,"mobile.customer.cancel.btn"
+42. Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+43. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+44. Click Continue,tap,,"mobile.customer.continue.btn"
+45. Enter OTP,type,123456,"mobile.customer.otp_input"
+46. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+47. Click Finish,tap,,"mobile.customer.finish.btn"
+48. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+49. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+50. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+51. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+52. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+53. Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+54. Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+55. Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+56. Click Confirm,tap,,"mobile.customer.confirm.btn"
+57. Wait For Ride,wait,5000,
+58. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+59. Ride Now,tap,,"mobile.customer.ride_now.btn"
+60. Load Driver App,switch_to,driver,
+61. Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+62. Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+63. Load User App,switch_to,user,
+64. Wait for OTP Layout to Load,wait_until_visible,,"mobile.customer.otp_display_element"
+65. Extract OTP from Screen,store_text,ride_otp,"mobile.customer.otp_display_element"
+66. Wait for load,wait,2000,
+67. Click SOS button,tap,,"mobile.customer.ride.sos_btn"
+68.Wait For Popup,wait,3000,
+69. Click Police bttuon,tap,,"mobile.customer.ride.sos_btn.police_btn"
+70. Click Call Button,tap,,"mobile.customer.ride.sos_btn.police.call_btn"
+71. Wait for reload the screen,wait,6000,
+72. Load Customer Apps,switch_to,user
+73. Load Driver App,switch_to,driver,
+74. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+75. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+76. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+77. Ride Arrived,tap,,"mobile.driver.arrived.btn"
+78. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+79. Yes Arrived,tap,,"mobile.driver.yes.btn"
+80. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+81. Start Ride,tap,,"mobile.driver.start_ride.btn"
+82. wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+83. Enter  Extracted OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+84. Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+85. Start Ride Button,tap,,"mobile.driver.start.btn"
+86. wait for data,wait,3000,
+87. Click SOS Button,tap_coordinate ,972:1207,COORDINATE_MODE
+88.Wait For Popup,wait,3000,
+89. Click Police Button,tap,,"mobile.driver.ride.sos.call_108"
+90. Click Call Button,tap,,"mobile.driver.ride.sos.call_btn"
+91. Wait for Phone Dialer,wait,5000,
+92. Load User App,switch_to,driver,
+93. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+94. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+95. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+96. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+97. Load User App,switch_to,user,
+98. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+99. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+100. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+101. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+102. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+103. Give Review,tap,,"mobile.customer.give_review.btn"
+104. Give Rating,tap_coordinate,348:1619,
+105. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+106. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+107. Trip Finished,tap,,"mobile.customer.done.btn"
+108. Load Driver App,switch_to,driver,
+109. Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+110. Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+111. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+112. Confirm Payment,tap,,"mobile.driver.yes.btn"
+113. Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+114. Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+115. Wait For Rating,wait,2000,
+116. Give Rating,tap_coordinate,348:1545,
+117. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+118. Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+119. Click Complete Button,tap,,"mobile.driver.complete.btn"
+120. Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+121. Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+122. Switch To Web,switch_to,web,
+123. Click Dashboard,Click,,"web.global.menu.dashboard"
+124. Click Setting,click,,"admin.setting.sidebar.menu"
+125. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+126. Search name,type,{policeName},"admin.setting.panic_call.search_name"
+127.Wait For Load,wait,1000,
+128. Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
+129. Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
+130. Wait For Delete,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -948,4 +1223,102 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BF2064-1F4D-4DE7-9489-136A9D518A49}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="45.77734375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
108th Commit: Epic Five Completed
</commit_message>
<xml_diff>
--- a/EPIC_0005_Ride_Safety_Calls.xlsx
+++ b/EPIC_0005_Ride_Safety_Calls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66346BB1-D980-40E5-BC74-7E1A9DFEFE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA09093-C24C-41B6-9D53-2F8A5FA003D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -686,6 +686,200 @@
 128. Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
 129. Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
 130. Wait For Delete,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3.  Switch To Web Session,switch_to,web,
+4. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5. Click drivers menu,click,,"admin.drivers.menu.icon"
+6. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+7. Verify Add Driver,verify,,"admin.drivers.add_page.header"
+8. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+9. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+10.Click Driver Type Dropdown,click,,"admin.drivers.driver_type.dropdown"
+11.Select pilot Option,click,,"admin.drivers.driver_type.dropdown_pilot"
+12. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+13. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+14. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+15. Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+16. Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+17. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+18. Select Source,click,,"admin.drivers.source_dropdown.select"
+19. Select Instagram,click,,"admin.drivers.instagram_option.span"
+20. Select Male Gender, click, , "admin.drivers.male_gender.div"
+21. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+22. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+23. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+24. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+25. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+26. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+27. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+28. Enter Bank Location, type, PARK STREET, "admin.drivers.banklocation.input"
+29. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+30. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+31. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+32. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+33. Click Submit, click, , "web.global.action.submit"
+34. Verify Driver Added, verify,, "web.global.toast.success"
+35. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click drivers menu,click,,"admin.drivers.menu.icon"
+37. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+38. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+39. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+40. Click Doc Icon,click,,"admin.drivers.docs.icon"
+41. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+42. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+43. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+44. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+45. Enter Expiry Date,set_date,2026-12-12,"admin.drivers.doc_expiry.input"
+46. Click Submit, click, , "web.global.action.submit"
+47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+48. Click Approve Driver,click,,"admin.drivers.docs.approval"
+49. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+50. Click Dashboard,click,,"web.global.menu.dashboard"
+51. Click drivers menu,click,,"admin.drivers.menu.icon"
+52. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+53. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+54. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+55.Wait For Load,wait,2000,
+56.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
+57.Click Wallet,click,,"admin.drivers.wallet.btn"
+58.Click Manage Transaction,click,,"admin.drivers.wallet.manage_transaction.btn"
+59.Enter Wallet Amout,type,500,"admin.drivers.wallet.wallet_amount_input"
+60.Click Dropdown,click,,"admin.drivers.wallet.option_dropdown"
+61.Select Add Money Optin,click,,"admin.drivers.wallet.option_add_money"
+62.Click Submit Button,click,,"admin.drivers.wallet.submit.btn"
+63.Wait For Recharge,wait,2000,
+64. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+65.Click Customer Icon,click,,"admin.menu.customer_icon"
+66.Click Add Customers,click,,"admin.menu.add_customers"
+67.Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
+68.Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+69.Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+70.Enter Contact Number,type,{randomPhone}&gt;&gt;customerPhone,"admin.customer.input_phone"
+71.Enter Emergency Number,type,{randomPhone},"admin.customer.input_Emergency_phone"
+72.Open Gender,click,,"admin.customer.dropdown_gender"
+73.Select Male,click,,"admin.customer.select_gender_male"
+74.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+75.Click Submit,click,,"web.global.action.submit"
+76.Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+77.Click Dashboard,click,,"web.global.menu.dashboard"
+78.Click Customer Icon,click,,"admin.menu.customer_icon"
+79.Click Verified Customers,click,,"admin.menu.verified_customers"
+80.Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+81.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+82.Wait For Load,wait,2000,
+83. Click Dashboard,Click,,"web.global.menu.dashboard"
+84.Click Setting,click,,"admin.setting.sidebar.menu"
+85.Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+86.Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
+87.Enter name,type,Police{randomAlpha}&gt;&gt;policeName,"admin.setting.panic_call.name_input"
+88.Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
+89.Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
+90.Contact number,type,100,"admin.setting.panic_call.contact_number"
+91.Select Status button,click,,"admin.setting.panic_call.status_dropdown"
+92.Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
+93.Submit button,click,,"web.global.action.submit"
+94.Search name,type,{policeName},"admin.setting.panic_call.search_name"
+95.Wait For Load,wait,1000,
+96. Load Driver App,switch_to,driver,
+97. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+98. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+99. Click Agree,tap,,"mobile.driver.agree.btn"
+100. Click Get Started,tap,,"mobile.driver.get_started.btn"
+101.Click Next,tap,,"mobile.driver.next.btn"
+102.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+103.Click Close,tap,,"mobile.driver.cancel.btn"
+104. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+105.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+106.Click Continue,tap,,"mobile.driver.continue.btn"
+107.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+108.Enter Account Holder,type,{autoName},"mobile.driver.bank_details.account_holder_name"
+109.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+110.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+111.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+112.Wait For Keyboard Minimises,hide_keyboard,,
+113.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+114.Wait For Keyboard Minimises,hide_keyboard,,
+115.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+116.Force Driver Location To Perambur,set_location,13.121030;80.232578,
+117.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+118.Wait for Toast to Hide,wait,3000,,
+119.Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+120.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+121.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+122.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+123. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+124. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+125.Wait For Hamburger Menu,wait,3000
+126.Click Online Toggle,tap_coordinate ,975:1935,COORDINATE_MODE
+126. Load User App,switch_to,user,
+127. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+128.Click Get Started,tap,,"mobile.customer.get_started.btn"
+129.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+130.Force User Location To Perambur,set_location,13.121030;80.232578,
+131.Click Next,tap,,"mobile.customer.next.btn"
+132.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+133.Click Close,tap,,"mobile.customer.cancel.btn"
+134.Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+135.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+136.Click Continue,tap,,"mobile.customer.continue.btn"
+137.Enter OTP,type,123456,"mobile.customer.otp_input"
+138.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+139.Click Finish,tap,,"mobile.customer.finish.btn"
+140.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+141.Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+142.Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+143.Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+144.Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+145.Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+146.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+147.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+148.Click Confirm,tap,,"mobile.customer.confirm.btn"
+149.Wait For Ride,wait,5000,
+150.Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+151.Ride Now,tap,,"mobile.customer.ride_now.btn"
+152.Load Driver App,switch_to,driver,
+153.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+154.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+155.Load User App,switch_to,user,
+156.Wait for OTP Layout to Load,wait_until_visible,,"mobile.customer.otp_display_element"
+157.Extract OTP from Screen,store_text,ride_otp,"mobile.customer.otp_display_element"
+158.Wait for load,wait,2000,
+159.Click SOS button,tap,,"mobile.customer.ride.sos_btn"
+160.Wait For Popup,wait,3000,
+161.Click Police bttuon,tap,,"mobile.customer.ride.sos_btn.police_btn"
+162.Click Call Button,tap,,"mobile.customer.ride.sos_btn.police.call_btn"
+163.Wait for Call Placement,wait,3000,
+164. Load Driver App,switch_to,driver,
+165.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+166.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+167.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+168.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+169.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+170.Yes Arrived,tap,,"mobile.driver.yes.btn"
+171.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+172.Start Ride,tap,,"mobile.driver.start_ride.btn"
+173.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+174.Enter  Extracted OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+175.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+176.Start Ride Button,tap,,"mobile.driver.start.btn"
+177.wait for data,wait,3000,
+178.Click SOS Button,tap_coordinate ,972:1207,COORDINATE_MODE
+179.Wait For Popup,wait,3000,
+180.Click Police Button,tap,,"mobile.driver.ride.sos.call_108"
+181.Click Call Button,tap,,"mobile.driver.ride.sos.call_btn"
+182.Wait for Phone Dialer,wait,3000,
+183. Switch To Web,switch_to,web,
+184. Click Dashboard,Click,,"web.global.menu.dashboard"
+185. Click Setting,click,,"admin.setting.sidebar.menu"
+186. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+187. Search name,type,{policeName},"admin.setting.panic_call.search_name"
+188.Wait For Load,wait,1000,
+189. Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
+190. Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
+191. Wait For Delete,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -1238,8 +1432,8 @@
     <col min="6" max="6" width="45.77734375" customWidth="1"/>
     <col min="7" max="7" width="71.44140625" customWidth="1"/>
     <col min="8" max="8" width="40.44140625" customWidth="1"/>
-    <col min="9" max="9" width="61.88671875" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+    <col min="9" max="9" width="34.21875" customWidth="1"/>
+    <col min="10" max="10" width="60.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1294,7 +1488,7 @@
         <v>32</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -1302,7 +1496,9 @@
       <c r="I2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
113th Commit: Data Cleanup Sheet Added
</commit_message>
<xml_diff>
--- a/EPIC_0005_Ride_Safety_Calls.xlsx
+++ b/EPIC_0005_Ride_Safety_Calls.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344E7EDC-4E79-4F21-8C02-658F12A79A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D588010-118B-45A9-9005-81CA1A9EDA39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
     <sheet name="CustomerAppEmergencyNumber" sheetId="48" r:id="rId2"/>
     <sheet name="PanicCallCheck" sheetId="49" r:id="rId3"/>
     <sheet name="RideAerialViewEarningReports" sheetId="50" r:id="rId4"/>
+    <sheet name="DataCleanUpSheet" sheetId="51" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1707,12 +1708,158 @@
 317.Wait For Loading,wait,4000,
 </t>
   </si>
+  <si>
+    <t>Pre-production</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>SA_TS_29</t>
+  </si>
+  <si>
+    <t>Clean The Test Data Created During Test Run</t>
+  </si>
+  <si>
+    <t>TC_SA_03_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
+  </si>
+  <si>
+    <t>No Manual Test Cases Since this is a data cleanup sheet after test execution</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CRITICAL SYSTEM WARNING: DATABASE INTEGRITY PROTOCOL</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-----------------------------------------</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">This sheet contains SQL Hooks that execute directly against the we1 Production/Staging database. DO NOT modify the SQL syntax, remove variable placeholders (e.g., {areaName}), or edit the WHERE clauses.
+Unauthorized changes may result in irreversible data loss or database corruption. If modifications are required, please contact the Automation Lead or the Database Administrator.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSWORD TO EDIT SHEET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> :eit6190
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet: SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_RG_05_test_data_cleanup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Remove  Subscrption Plan,sql delete,,"DELETE FROM we1.panic_call WHERE name = '{policeName}';"
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1732,6 +1879,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1763,7 +1918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1776,6 +1931,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2450,4 +2615,92 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FCA0D8B-8968-4717-A6E5-49959BF0DAC0}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
+    <col min="5" max="6" width="34.109375" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
+    <col min="8" max="8" width="31.77734375" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="8"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>